<commit_message>
Fija confirmación de correo PKCE con sesión previa: preserva code verifier al cerrar pestaña web y avisa si el enlace falla
</commit_message>
<xml_diff>
--- a/docs/Pruebas manuales/Pruebas_manuales_01-04.xlsx
+++ b/docs/Pruebas manuales/Pruebas_manuales_01-04.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jaime\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\esteticaybellezastrani\docs\Pruebas manuales\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0112A99-316A-4F10-9D50-D1E27D84675B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1DCB15D3-0FD2-4E01-9F1E-F8C36CAC1621}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2784" yWindow="1488" windowWidth="18552" windowHeight="10428" activeTab="1" xr2:uid="{FC97818C-F504-4FE2-93BA-77FDB8B1BF19}"/>
+    <workbookView xWindow="1650" yWindow="645" windowWidth="18750" windowHeight="10875" activeTab="1" xr2:uid="{FC97818C-F504-4FE2-93BA-77FDB8B1BF19}"/>
   </bookViews>
   <sheets>
     <sheet name="Como_evaluar" sheetId="5" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1097" uniqueCount="694">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1123" uniqueCount="695">
   <si>
     <t>Pruebas manuales — auth_users</t>
   </si>
@@ -2112,26 +2112,29 @@
     <t>7. Cierra el documento: totales por prioridad y resultado, % de pase y lista de fallas que bloquean el release.</t>
   </si>
   <si>
-    <t>Falla, Phone=NULL</t>
-  </si>
-  <si>
-    <t>Falla, no envia confirmación ni correo</t>
-  </si>
-  <si>
-    <t>Falla, datos generados sin autenticar email, sin Phone. Al hacer Login: paciente no existe. Trata de registrar, usuario ya existe.</t>
-  </si>
-  <si>
-    <t>Falla. No se pudo cargar perfil de especialista.</t>
-  </si>
-  <si>
-    <t>Falla. Perfil no encontrado, contacta a soporte.</t>
+    <t>Falla, Phone en Users= NULL</t>
+  </si>
+  <si>
+    <t>Chrome may soon delete state for intermediate websites in a recent navigation chain</t>
+  </si>
+  <si>
+    <t>Id no debe mostrarse, sólo por ahora para pruebas. Debe dejar seleccionar algún Avatar.</t>
+  </si>
+  <si>
+    <t>Pasa a confirmación email sin error de validación.</t>
+  </si>
+  <si>
+    <t>Error en Ingles. Invalid Login Credentials. Debe explicar el error dependiendo la región del sistema.</t>
+  </si>
+  <si>
+    <t>Sin forma de regresar a vista anterior</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2154,6 +2157,12 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color rgb="FFDEE4E4"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="3">
@@ -2182,7 +2191,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -2200,6 +2209,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2535,36 +2545,36 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4A2BE10C-6C1D-4B18-9540-EA2518AD06EA}">
   <dimension ref="A1:C27"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="18.6640625" customWidth="1"/>
-    <col min="2" max="2" width="90.6640625" customWidth="1"/>
-    <col min="3" max="3" width="60.6640625" customWidth="1"/>
+    <col min="1" max="1" width="18.7109375" customWidth="1"/>
+    <col min="2" max="2" width="90.7109375" customWidth="1"/>
+    <col min="3" max="3" width="60.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="18" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>657</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>658</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="8" t="s">
         <v>659</v>
       </c>
       <c r="B4" s="8"/>
       <c r="C4" s="8"/>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>660</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
         <v>14</v>
       </c>
@@ -2572,7 +2582,7 @@
         <v>661</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>662</v>
       </c>
@@ -2580,7 +2590,7 @@
         <v>663</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>664</v>
       </c>
@@ -2588,7 +2598,7 @@
         <v>665</v>
       </c>
     </row>
-    <row r="10" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>380</v>
       </c>
@@ -2596,7 +2606,7 @@
         <v>666</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>667</v>
       </c>
@@ -2604,12 +2614,12 @@
         <v>668</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
         <v>669</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" s="4" t="s">
         <v>670</v>
       </c>
@@ -2620,7 +2630,7 @@
         <v>672</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A15" s="7" t="s">
         <v>27</v>
       </c>
@@ -2631,7 +2641,7 @@
         <v>674</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" s="7" t="s">
         <v>53</v>
       </c>
@@ -2642,7 +2652,7 @@
         <v>676</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" s="7" t="s">
         <v>22</v>
       </c>
@@ -2653,7 +2663,7 @@
         <v>678</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" s="7" t="s">
         <v>183</v>
       </c>
@@ -2664,54 +2674,54 @@
         <v>680</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
         <v>681</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" s="8" t="s">
         <v>682</v>
       </c>
       <c r="B21" s="8"/>
       <c r="C21" s="8"/>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" s="8" t="s">
         <v>683</v>
       </c>
       <c r="B22" s="8"/>
       <c r="C22" s="8"/>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" s="8" t="s">
         <v>684</v>
       </c>
       <c r="B23" s="8"/>
       <c r="C23" s="8"/>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" s="8" t="s">
         <v>685</v>
       </c>
       <c r="B24" s="8"/>
       <c r="C24" s="8"/>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" s="8" t="s">
         <v>686</v>
       </c>
       <c r="B25" s="8"/>
       <c r="C25" s="8"/>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" s="8" t="s">
         <v>687</v>
       </c>
       <c r="B26" s="8"/>
       <c r="C26" s="8"/>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" s="8" t="s">
         <v>688</v>
       </c>
@@ -2736,24 +2746,24 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7B31A8B7-D028-4D4D-885E-7030DE451177}">
   <dimension ref="A1:I56"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="14.6640625" customWidth="1"/>
-    <col min="2" max="2" width="15.5546875" customWidth="1"/>
-    <col min="3" max="3" width="26.88671875" customWidth="1"/>
-    <col min="4" max="4" width="20.33203125" customWidth="1"/>
-    <col min="5" max="6" width="42.6640625" customWidth="1"/>
-    <col min="7" max="7" width="10.6640625" customWidth="1"/>
-    <col min="8" max="8" width="12.6640625" customWidth="1"/>
-    <col min="9" max="9" width="30.6640625" customWidth="1"/>
+    <col min="1" max="1" width="14.7109375" customWidth="1"/>
+    <col min="2" max="2" width="15.5703125" customWidth="1"/>
+    <col min="3" max="3" width="26.85546875" customWidth="1"/>
+    <col min="4" max="4" width="20.28515625" customWidth="1"/>
+    <col min="5" max="6" width="42.7109375" customWidth="1"/>
+    <col min="7" max="7" width="10.7109375" customWidth="1"/>
+    <col min="8" max="8" width="18" customWidth="1"/>
+    <col min="9" max="9" width="30.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="18" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:9" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
@@ -2761,7 +2771,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>3</v>
       </c>
@@ -2769,7 +2779,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>5</v>
       </c>
@@ -2777,7 +2787,7 @@
         <v>46248</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>6</v>
       </c>
@@ -2785,7 +2795,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
         <v>7</v>
       </c>
@@ -2814,7 +2824,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="8" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A8" s="5" t="s">
         <v>16</v>
       </c>
@@ -2836,12 +2846,11 @@
       <c r="G8" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="H8" s="5"/>
-      <c r="I8" s="5" t="s">
+      <c r="H8" s="5" t="s">
         <v>662</v>
       </c>
     </row>
-    <row r="9" spans="1:9" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A9" s="5" t="s">
         <v>23</v>
       </c>
@@ -2863,12 +2872,11 @@
       <c r="G9" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="H9" s="5"/>
-      <c r="I9" s="5" t="s">
+      <c r="H9" s="5" t="s">
         <v>689</v>
       </c>
     </row>
-    <row r="10" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" s="5" t="s">
         <v>28</v>
       </c>
@@ -2890,12 +2898,11 @@
       <c r="G10" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="H10" s="5"/>
-      <c r="I10" s="5" t="s">
-        <v>690</v>
-      </c>
-    </row>
-    <row r="11" spans="1:9" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="H10" s="5" t="s">
+        <v>662</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A11" s="5" t="s">
         <v>33</v>
       </c>
@@ -2917,12 +2924,11 @@
       <c r="G11" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="H11" s="5"/>
-      <c r="I11" s="5" t="s">
-        <v>691</v>
-      </c>
-    </row>
-    <row r="12" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="H11" s="5" t="s">
+        <v>662</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" s="5" t="s">
         <v>38</v>
       </c>
@@ -2944,12 +2950,11 @@
       <c r="G12" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="H12" s="5"/>
-      <c r="I12" s="5" t="s">
-        <v>692</v>
-      </c>
-    </row>
-    <row r="13" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="H12" s="5" t="s">
+        <v>662</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" s="5" t="s">
         <v>43</v>
       </c>
@@ -2971,12 +2976,11 @@
       <c r="G13" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="H13" s="5"/>
-      <c r="I13" s="5" t="s">
-        <v>693</v>
-      </c>
-    </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="H13" s="5" t="s">
+        <v>662</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A14" s="5" t="s">
         <v>48</v>
       </c>
@@ -2998,12 +3002,11 @@
       <c r="G14" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="H14" s="5"/>
-      <c r="I14" s="5" t="s">
+      <c r="H14" s="5" t="s">
         <v>662</v>
       </c>
     </row>
-    <row r="15" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A15" s="5" t="s">
         <v>54</v>
       </c>
@@ -3025,10 +3028,14 @@
       <c r="G15" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="H15" s="5"/>
-      <c r="I15" s="5"/>
-    </row>
-    <row r="16" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="H15" s="5" t="s">
+        <v>664</v>
+      </c>
+      <c r="I15" s="5" t="s">
+        <v>691</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A16" s="5" t="s">
         <v>59</v>
       </c>
@@ -3050,10 +3057,12 @@
       <c r="G16" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="H16" s="5"/>
+      <c r="H16" s="5" t="s">
+        <v>664</v>
+      </c>
       <c r="I16" s="5"/>
     </row>
-    <row r="17" spans="1:9" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:9" ht="75" x14ac:dyDescent="0.25">
       <c r="A17" s="5" t="s">
         <v>63</v>
       </c>
@@ -3075,10 +3084,14 @@
       <c r="G17" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="H17" s="5"/>
-      <c r="I17" s="5"/>
-    </row>
-    <row r="18" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="H17" s="5" t="s">
+        <v>664</v>
+      </c>
+      <c r="I17" s="9" t="s">
+        <v>690</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A18" s="5" t="s">
         <v>67</v>
       </c>
@@ -3100,10 +3113,12 @@
       <c r="G18" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="H18" s="5"/>
+      <c r="H18" s="5" t="s">
+        <v>662</v>
+      </c>
       <c r="I18" s="5"/>
     </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A19" s="5" t="s">
         <v>71</v>
       </c>
@@ -3125,10 +3140,12 @@
       <c r="G19" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="H19" s="5"/>
+      <c r="H19" s="5" t="s">
+        <v>662</v>
+      </c>
       <c r="I19" s="5"/>
     </row>
-    <row r="20" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A20" s="5" t="s">
         <v>75</v>
       </c>
@@ -3150,10 +3167,14 @@
       <c r="G20" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="H20" s="5"/>
-      <c r="I20" s="5"/>
-    </row>
-    <row r="21" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="H20" s="5" t="s">
+        <v>662</v>
+      </c>
+      <c r="I20" s="5" t="s">
+        <v>693</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A21" s="5" t="s">
         <v>81</v>
       </c>
@@ -3175,10 +3196,14 @@
       <c r="G21" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="H21" s="5"/>
-      <c r="I21" s="5"/>
-    </row>
-    <row r="22" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="H21" s="5" t="s">
+        <v>662</v>
+      </c>
+      <c r="I21" s="5" t="s">
+        <v>693</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A22" s="5" t="s">
         <v>85</v>
       </c>
@@ -3200,10 +3225,14 @@
       <c r="G22" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="H22" s="5"/>
-      <c r="I22" s="5"/>
-    </row>
-    <row r="23" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="H22" s="5" t="s">
+        <v>662</v>
+      </c>
+      <c r="I22" s="5" t="s">
+        <v>693</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A23" s="5" t="s">
         <v>89</v>
       </c>
@@ -3225,10 +3254,14 @@
       <c r="G23" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="H23" s="5"/>
-      <c r="I23" s="5"/>
-    </row>
-    <row r="24" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="H23" s="5" t="s">
+        <v>664</v>
+      </c>
+      <c r="I23" s="5" t="s">
+        <v>692</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A24" s="5" t="s">
         <v>94</v>
       </c>
@@ -3250,10 +3283,14 @@
       <c r="G24" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="H24" s="5"/>
-      <c r="I24" s="5"/>
-    </row>
-    <row r="25" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="H24" s="5" t="s">
+        <v>662</v>
+      </c>
+      <c r="I24" s="5" t="s">
+        <v>693</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A25" s="5" t="s">
         <v>98</v>
       </c>
@@ -3275,10 +3312,14 @@
       <c r="G25" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="H25" s="5"/>
-      <c r="I25" s="5"/>
-    </row>
-    <row r="26" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="H25" s="5" t="s">
+        <v>662</v>
+      </c>
+      <c r="I25" s="5" t="s">
+        <v>693</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A26" s="5" t="s">
         <v>103</v>
       </c>
@@ -3303,7 +3344,7 @@
       <c r="H26" s="5"/>
       <c r="I26" s="5"/>
     </row>
-    <row r="27" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A27" s="5" t="s">
         <v>108</v>
       </c>
@@ -3328,7 +3369,7 @@
       <c r="H27" s="5"/>
       <c r="I27" s="5"/>
     </row>
-    <row r="28" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A28" s="5" t="s">
         <v>112</v>
       </c>
@@ -3353,7 +3394,7 @@
       <c r="H28" s="5"/>
       <c r="I28" s="5"/>
     </row>
-    <row r="29" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A29" s="5" t="s">
         <v>115</v>
       </c>
@@ -3378,7 +3419,7 @@
       <c r="H29" s="5"/>
       <c r="I29" s="5"/>
     </row>
-    <row r="30" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A30" s="5" t="s">
         <v>118</v>
       </c>
@@ -3403,7 +3444,7 @@
       <c r="H30" s="5"/>
       <c r="I30" s="5"/>
     </row>
-    <row r="31" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A31" s="5" t="s">
         <v>122</v>
       </c>
@@ -3425,10 +3466,12 @@
       <c r="G31" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="H31" s="5"/>
+      <c r="H31" s="5" t="s">
+        <v>662</v>
+      </c>
       <c r="I31" s="5"/>
     </row>
-    <row r="32" spans="1:9" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A32" s="5" t="s">
         <v>127</v>
       </c>
@@ -3450,10 +3493,12 @@
       <c r="G32" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="H32" s="5"/>
+      <c r="H32" s="5" t="s">
+        <v>662</v>
+      </c>
       <c r="I32" s="5"/>
     </row>
-    <row r="33" spans="1:9" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A33" s="5" t="s">
         <v>132</v>
       </c>
@@ -3475,10 +3520,12 @@
       <c r="G33" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="H33" s="5"/>
+      <c r="H33" s="5" t="s">
+        <v>662</v>
+      </c>
       <c r="I33" s="5"/>
     </row>
-    <row r="34" spans="1:9" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A34" s="5" t="s">
         <v>135</v>
       </c>
@@ -3503,7 +3550,7 @@
       <c r="H34" s="5"/>
       <c r="I34" s="5"/>
     </row>
-    <row r="35" spans="1:9" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A35" s="5" t="s">
         <v>139</v>
       </c>
@@ -3528,7 +3575,7 @@
       <c r="H35" s="5"/>
       <c r="I35" s="5"/>
     </row>
-    <row r="36" spans="1:9" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A36" s="5" t="s">
         <v>143</v>
       </c>
@@ -3553,7 +3600,7 @@
       <c r="H36" s="5"/>
       <c r="I36" s="5"/>
     </row>
-    <row r="37" spans="1:9" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A37" s="5" t="s">
         <v>147</v>
       </c>
@@ -3578,7 +3625,7 @@
       <c r="H37" s="5"/>
       <c r="I37" s="5"/>
     </row>
-    <row r="38" spans="1:9" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A38" s="5" t="s">
         <v>150</v>
       </c>
@@ -3603,7 +3650,7 @@
       <c r="H38" s="5"/>
       <c r="I38" s="5"/>
     </row>
-    <row r="39" spans="1:9" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A39" s="5" t="s">
         <v>154</v>
       </c>
@@ -3628,7 +3675,7 @@
       <c r="H39" s="5"/>
       <c r="I39" s="5"/>
     </row>
-    <row r="40" spans="1:9" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A40" s="5" t="s">
         <v>159</v>
       </c>
@@ -3653,7 +3700,7 @@
       <c r="H40" s="5"/>
       <c r="I40" s="5"/>
     </row>
-    <row r="41" spans="1:9" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A41" s="5" t="s">
         <v>164</v>
       </c>
@@ -3680,7 +3727,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="42" spans="1:9" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A42" s="5" t="s">
         <v>170</v>
       </c>
@@ -3705,7 +3752,7 @@
       <c r="H42" s="5"/>
       <c r="I42" s="5"/>
     </row>
-    <row r="43" spans="1:9" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A43" s="5" t="s">
         <v>174</v>
       </c>
@@ -3730,7 +3777,7 @@
       <c r="H43" s="5"/>
       <c r="I43" s="5"/>
     </row>
-    <row r="44" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A44" s="5" t="s">
         <v>179</v>
       </c>
@@ -3752,10 +3799,14 @@
       <c r="G44" s="5" t="s">
         <v>183</v>
       </c>
-      <c r="H44" s="5"/>
-      <c r="I44" s="5"/>
-    </row>
-    <row r="45" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="H44" s="5" t="s">
+        <v>662</v>
+      </c>
+      <c r="I44" s="5" t="s">
+        <v>694</v>
+      </c>
+    </row>
+    <row r="45" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A45" s="5" t="s">
         <v>184</v>
       </c>
@@ -3780,7 +3831,7 @@
       <c r="H45" s="5"/>
       <c r="I45" s="5"/>
     </row>
-    <row r="46" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A46" s="5" t="s">
         <v>189</v>
       </c>
@@ -3805,7 +3856,7 @@
       <c r="H46" s="5"/>
       <c r="I46" s="5"/>
     </row>
-    <row r="47" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A47" s="5" t="s">
         <v>194</v>
       </c>
@@ -3830,7 +3881,7 @@
       <c r="H47" s="5"/>
       <c r="I47" s="5"/>
     </row>
-    <row r="48" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A48" s="5" t="s">
         <v>198</v>
       </c>
@@ -3855,7 +3906,7 @@
       <c r="H48" s="5"/>
       <c r="I48" s="5"/>
     </row>
-    <row r="49" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A49" s="5" t="s">
         <v>204</v>
       </c>
@@ -3880,7 +3931,7 @@
       <c r="H49" s="5"/>
       <c r="I49" s="5"/>
     </row>
-    <row r="50" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A50" s="5" t="s">
         <v>208</v>
       </c>
@@ -3902,10 +3953,12 @@
       <c r="G50" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="H50" s="5"/>
+      <c r="H50" s="5" t="s">
+        <v>662</v>
+      </c>
       <c r="I50" s="5"/>
     </row>
-    <row r="51" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A51" s="5" t="s">
         <v>213</v>
       </c>
@@ -3930,7 +3983,7 @@
       <c r="H51" s="5"/>
       <c r="I51" s="5"/>
     </row>
-    <row r="52" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A52" s="5" t="s">
         <v>217</v>
       </c>
@@ -3955,7 +4008,7 @@
       <c r="H52" s="5"/>
       <c r="I52" s="5"/>
     </row>
-    <row r="53" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A53" s="5" t="s">
         <v>220</v>
       </c>
@@ -3980,7 +4033,7 @@
       <c r="H53" s="5"/>
       <c r="I53" s="5"/>
     </row>
-    <row r="54" spans="1:9" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A54" s="5" t="s">
         <v>225</v>
       </c>
@@ -4002,10 +4055,12 @@
       <c r="G54" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="H54" s="5"/>
+      <c r="H54" s="5" t="s">
+        <v>662</v>
+      </c>
       <c r="I54" s="5"/>
     </row>
-    <row r="55" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A55" s="5" t="s">
         <v>231</v>
       </c>
@@ -4030,7 +4085,7 @@
       <c r="H55" s="5"/>
       <c r="I55" s="5"/>
     </row>
-    <row r="56" spans="1:9" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A56" s="5" t="s">
         <v>236</v>
       </c>
@@ -4063,24 +4118,24 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F33AE011-15CC-4821-A161-FEC86D683C66}">
   <dimension ref="A1:I51"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="8.5546875" customWidth="1"/>
-    <col min="2" max="2" width="15.44140625" customWidth="1"/>
-    <col min="3" max="3" width="24.44140625" customWidth="1"/>
-    <col min="4" max="4" width="27.88671875" customWidth="1"/>
-    <col min="5" max="6" width="42.6640625" customWidth="1"/>
-    <col min="7" max="7" width="10.6640625" customWidth="1"/>
-    <col min="8" max="8" width="12.6640625" customWidth="1"/>
-    <col min="9" max="9" width="30.6640625" customWidth="1"/>
+    <col min="1" max="1" width="8.5703125" customWidth="1"/>
+    <col min="2" max="2" width="15.42578125" customWidth="1"/>
+    <col min="3" max="3" width="24.42578125" customWidth="1"/>
+    <col min="4" max="4" width="27.85546875" customWidth="1"/>
+    <col min="5" max="6" width="42.7109375" customWidth="1"/>
+    <col min="7" max="7" width="10.7109375" customWidth="1"/>
+    <col min="8" max="8" width="12.7109375" customWidth="1"/>
+    <col min="9" max="9" width="30.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="18" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:9" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>241</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
@@ -4088,7 +4143,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>3</v>
       </c>
@@ -4096,7 +4151,7 @@
         <v>243</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>5</v>
       </c>
@@ -4104,7 +4159,7 @@
         <v>46248</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>6</v>
       </c>
@@ -4112,7 +4167,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
         <v>7</v>
       </c>
@@ -4141,7 +4196,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="8" spans="1:9" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A8" s="5" t="s">
         <v>244</v>
       </c>
@@ -4166,7 +4221,7 @@
       <c r="H8" s="5"/>
       <c r="I8" s="5"/>
     </row>
-    <row r="9" spans="1:9" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A9" s="5" t="s">
         <v>249</v>
       </c>
@@ -4191,7 +4246,7 @@
       <c r="H9" s="5"/>
       <c r="I9" s="5"/>
     </row>
-    <row r="10" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A10" s="5" t="s">
         <v>254</v>
       </c>
@@ -4216,7 +4271,7 @@
       <c r="H10" s="5"/>
       <c r="I10" s="5"/>
     </row>
-    <row r="11" spans="1:9" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A11" s="5" t="s">
         <v>259</v>
       </c>
@@ -4241,7 +4296,7 @@
       <c r="H11" s="5"/>
       <c r="I11" s="5"/>
     </row>
-    <row r="12" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A12" s="5" t="s">
         <v>263</v>
       </c>
@@ -4266,7 +4321,7 @@
       <c r="H12" s="5"/>
       <c r="I12" s="5"/>
     </row>
-    <row r="13" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A13" s="5" t="s">
         <v>268</v>
       </c>
@@ -4291,7 +4346,7 @@
       <c r="H13" s="5"/>
       <c r="I13" s="5"/>
     </row>
-    <row r="14" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A14" s="5" t="s">
         <v>273</v>
       </c>
@@ -4316,7 +4371,7 @@
       <c r="H14" s="5"/>
       <c r="I14" s="5"/>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A15" s="5" t="s">
         <v>278</v>
       </c>
@@ -4341,7 +4396,7 @@
       <c r="H15" s="5"/>
       <c r="I15" s="5"/>
     </row>
-    <row r="16" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A16" s="5" t="s">
         <v>282</v>
       </c>
@@ -4366,7 +4421,7 @@
       <c r="H16" s="5"/>
       <c r="I16" s="5"/>
     </row>
-    <row r="17" spans="1:9" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A17" s="5" t="s">
         <v>287</v>
       </c>
@@ -4391,7 +4446,7 @@
       <c r="H17" s="5"/>
       <c r="I17" s="5"/>
     </row>
-    <row r="18" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A18" s="5" t="s">
         <v>291</v>
       </c>
@@ -4416,7 +4471,7 @@
       <c r="H18" s="5"/>
       <c r="I18" s="5"/>
     </row>
-    <row r="19" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A19" s="5" t="s">
         <v>296</v>
       </c>
@@ -4441,7 +4496,7 @@
       <c r="H19" s="5"/>
       <c r="I19" s="5"/>
     </row>
-    <row r="20" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A20" s="5" t="s">
         <v>301</v>
       </c>
@@ -4466,7 +4521,7 @@
       <c r="H20" s="5"/>
       <c r="I20" s="5"/>
     </row>
-    <row r="21" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A21" s="5" t="s">
         <v>305</v>
       </c>
@@ -4491,7 +4546,7 @@
       <c r="H21" s="5"/>
       <c r="I21" s="5"/>
     </row>
-    <row r="22" spans="1:9" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A22" s="5" t="s">
         <v>310</v>
       </c>
@@ -4516,7 +4571,7 @@
       <c r="H22" s="5"/>
       <c r="I22" s="5"/>
     </row>
-    <row r="23" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A23" s="5" t="s">
         <v>314</v>
       </c>
@@ -4541,7 +4596,7 @@
       <c r="H23" s="5"/>
       <c r="I23" s="5"/>
     </row>
-    <row r="24" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A24" s="5" t="s">
         <v>319</v>
       </c>
@@ -4566,7 +4621,7 @@
       <c r="H24" s="5"/>
       <c r="I24" s="5"/>
     </row>
-    <row r="25" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A25" s="5" t="s">
         <v>324</v>
       </c>
@@ -4591,7 +4646,7 @@
       <c r="H25" s="5"/>
       <c r="I25" s="5"/>
     </row>
-    <row r="26" spans="1:9" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A26" s="5" t="s">
         <v>329</v>
       </c>
@@ -4616,7 +4671,7 @@
       <c r="H26" s="5"/>
       <c r="I26" s="5"/>
     </row>
-    <row r="27" spans="1:9" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A27" s="5" t="s">
         <v>332</v>
       </c>
@@ -4641,7 +4696,7 @@
       <c r="H27" s="5"/>
       <c r="I27" s="5"/>
     </row>
-    <row r="28" spans="1:9" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:9" ht="75" x14ac:dyDescent="0.25">
       <c r="A28" s="5" t="s">
         <v>335</v>
       </c>
@@ -4666,7 +4721,7 @@
       <c r="H28" s="5"/>
       <c r="I28" s="5"/>
     </row>
-    <row r="29" spans="1:9" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A29" s="5" t="s">
         <v>340</v>
       </c>
@@ -4691,7 +4746,7 @@
       <c r="H29" s="5"/>
       <c r="I29" s="5"/>
     </row>
-    <row r="30" spans="1:9" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A30" s="5" t="s">
         <v>344</v>
       </c>
@@ -4716,7 +4771,7 @@
       <c r="H30" s="5"/>
       <c r="I30" s="5"/>
     </row>
-    <row r="31" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A31" s="5" t="s">
         <v>349</v>
       </c>
@@ -4741,7 +4796,7 @@
       <c r="H31" s="5"/>
       <c r="I31" s="5"/>
     </row>
-    <row r="32" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A32" s="5" t="s">
         <v>353</v>
       </c>
@@ -4766,7 +4821,7 @@
       <c r="H32" s="5"/>
       <c r="I32" s="5"/>
     </row>
-    <row r="33" spans="1:9" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A33" s="5" t="s">
         <v>357</v>
       </c>
@@ -4791,7 +4846,7 @@
       <c r="H33" s="5"/>
       <c r="I33" s="5"/>
     </row>
-    <row r="34" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A34" s="5" t="s">
         <v>361</v>
       </c>
@@ -4816,7 +4871,7 @@
       <c r="H34" s="5"/>
       <c r="I34" s="5"/>
     </row>
-    <row r="35" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A35" s="5" t="s">
         <v>365</v>
       </c>
@@ -4841,7 +4896,7 @@
       <c r="H35" s="5"/>
       <c r="I35" s="5"/>
     </row>
-    <row r="36" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A36" s="5" t="s">
         <v>370</v>
       </c>
@@ -4866,7 +4921,7 @@
       <c r="H36" s="5"/>
       <c r="I36" s="5"/>
     </row>
-    <row r="37" spans="1:9" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A37" s="5" t="s">
         <v>374</v>
       </c>
@@ -4891,7 +4946,7 @@
       <c r="H37" s="5"/>
       <c r="I37" s="5"/>
     </row>
-    <row r="38" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A38" s="5" t="s">
         <v>379</v>
       </c>
@@ -4916,7 +4971,7 @@
       <c r="H38" s="5"/>
       <c r="I38" s="5"/>
     </row>
-    <row r="39" spans="1:9" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A39" s="5" t="s">
         <v>383</v>
       </c>
@@ -4941,7 +4996,7 @@
       <c r="H39" s="5"/>
       <c r="I39" s="5"/>
     </row>
-    <row r="40" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A40" s="5" t="s">
         <v>388</v>
       </c>
@@ -4966,7 +5021,7 @@
       <c r="H40" s="5"/>
       <c r="I40" s="5"/>
     </row>
-    <row r="41" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A41" s="5" t="s">
         <v>392</v>
       </c>
@@ -4991,7 +5046,7 @@
       <c r="H41" s="5"/>
       <c r="I41" s="5"/>
     </row>
-    <row r="42" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A42" s="5" t="s">
         <v>396</v>
       </c>
@@ -5016,7 +5071,7 @@
       <c r="H42" s="5"/>
       <c r="I42" s="5"/>
     </row>
-    <row r="43" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A43" s="5" t="s">
         <v>400</v>
       </c>
@@ -5041,7 +5096,7 @@
       <c r="H43" s="5"/>
       <c r="I43" s="5"/>
     </row>
-    <row r="44" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A44" s="5" t="s">
         <v>404</v>
       </c>
@@ -5066,7 +5121,7 @@
       <c r="H44" s="5"/>
       <c r="I44" s="5"/>
     </row>
-    <row r="45" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A45" s="5" t="s">
         <v>409</v>
       </c>
@@ -5091,7 +5146,7 @@
       <c r="H45" s="5"/>
       <c r="I45" s="5"/>
     </row>
-    <row r="46" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A46" s="5" t="s">
         <v>414</v>
       </c>
@@ -5116,7 +5171,7 @@
       <c r="H46" s="5"/>
       <c r="I46" s="5"/>
     </row>
-    <row r="47" spans="1:9" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A47" s="5" t="s">
         <v>419</v>
       </c>
@@ -5141,7 +5196,7 @@
       <c r="H47" s="5"/>
       <c r="I47" s="5"/>
     </row>
-    <row r="48" spans="1:9" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A48" s="5" t="s">
         <v>424</v>
       </c>
@@ -5166,7 +5221,7 @@
       <c r="H48" s="5"/>
       <c r="I48" s="5"/>
     </row>
-    <row r="49" spans="1:9" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A49" s="5" t="s">
         <v>428</v>
       </c>
@@ -5191,7 +5246,7 @@
       <c r="H49" s="5"/>
       <c r="I49" s="5"/>
     </row>
-    <row r="50" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A50" s="5" t="s">
         <v>433</v>
       </c>
@@ -5216,7 +5271,7 @@
       <c r="H50" s="5"/>
       <c r="I50" s="5"/>
     </row>
-    <row r="51" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A51" s="5" t="s">
         <v>438</v>
       </c>
@@ -5249,24 +5304,24 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8714DB36-549F-44E5-8199-43729EDA2F34}">
   <dimension ref="A1:I36"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="14.6640625" customWidth="1"/>
-    <col min="2" max="2" width="26.6640625" customWidth="1"/>
-    <col min="3" max="3" width="30.6640625" customWidth="1"/>
-    <col min="4" max="4" width="32.6640625" customWidth="1"/>
-    <col min="5" max="6" width="42.6640625" customWidth="1"/>
-    <col min="7" max="7" width="10.6640625" customWidth="1"/>
-    <col min="8" max="8" width="12.6640625" customWidth="1"/>
-    <col min="9" max="9" width="30.6640625" customWidth="1"/>
+    <col min="1" max="1" width="14.7109375" customWidth="1"/>
+    <col min="2" max="2" width="26.7109375" customWidth="1"/>
+    <col min="3" max="3" width="30.7109375" customWidth="1"/>
+    <col min="4" max="4" width="32.7109375" customWidth="1"/>
+    <col min="5" max="6" width="42.7109375" customWidth="1"/>
+    <col min="7" max="7" width="10.7109375" customWidth="1"/>
+    <col min="8" max="8" width="12.7109375" customWidth="1"/>
+    <col min="9" max="9" width="30.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="18" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:9" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>443</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
@@ -5274,7 +5329,7 @@
         <v>444</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>3</v>
       </c>
@@ -5282,7 +5337,7 @@
         <v>445</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>5</v>
       </c>
@@ -5290,7 +5345,7 @@
         <v>46248</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>6</v>
       </c>
@@ -5298,7 +5353,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
         <v>7</v>
       </c>
@@ -5327,7 +5382,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="8" spans="1:9" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A8" s="5" t="s">
         <v>446</v>
       </c>
@@ -5352,7 +5407,7 @@
       <c r="H8" s="5"/>
       <c r="I8" s="5"/>
     </row>
-    <row r="9" spans="1:9" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A9" s="5" t="s">
         <v>451</v>
       </c>
@@ -5377,7 +5432,7 @@
       <c r="H9" s="5"/>
       <c r="I9" s="5"/>
     </row>
-    <row r="10" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A10" s="5" t="s">
         <v>455</v>
       </c>
@@ -5402,7 +5457,7 @@
       <c r="H10" s="5"/>
       <c r="I10" s="5"/>
     </row>
-    <row r="11" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A11" s="5" t="s">
         <v>459</v>
       </c>
@@ -5427,7 +5482,7 @@
       <c r="H11" s="5"/>
       <c r="I11" s="5"/>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" s="5" t="s">
         <v>463</v>
       </c>
@@ -5452,7 +5507,7 @@
       <c r="H12" s="5"/>
       <c r="I12" s="5"/>
     </row>
-    <row r="13" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A13" s="5" t="s">
         <v>468</v>
       </c>
@@ -5477,7 +5532,7 @@
       <c r="H13" s="5"/>
       <c r="I13" s="5"/>
     </row>
-    <row r="14" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A14" s="5" t="s">
         <v>473</v>
       </c>
@@ -5502,7 +5557,7 @@
       <c r="H14" s="5"/>
       <c r="I14" s="5"/>
     </row>
-    <row r="15" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A15" s="5" t="s">
         <v>477</v>
       </c>
@@ -5527,7 +5582,7 @@
       <c r="H15" s="5"/>
       <c r="I15" s="5"/>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" s="5" t="s">
         <v>482</v>
       </c>
@@ -5552,7 +5607,7 @@
       <c r="H16" s="5"/>
       <c r="I16" s="5"/>
     </row>
-    <row r="17" spans="1:9" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A17" s="5" t="s">
         <v>487</v>
       </c>
@@ -5577,7 +5632,7 @@
       <c r="H17" s="5"/>
       <c r="I17" s="5"/>
     </row>
-    <row r="18" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A18" s="5" t="s">
         <v>492</v>
       </c>
@@ -5602,7 +5657,7 @@
       <c r="H18" s="5"/>
       <c r="I18" s="5"/>
     </row>
-    <row r="19" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A19" s="5" t="s">
         <v>496</v>
       </c>
@@ -5627,7 +5682,7 @@
       <c r="H19" s="5"/>
       <c r="I19" s="5"/>
     </row>
-    <row r="20" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A20" s="5" t="s">
         <v>500</v>
       </c>
@@ -5652,7 +5707,7 @@
       <c r="H20" s="5"/>
       <c r="I20" s="5"/>
     </row>
-    <row r="21" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A21" s="5" t="s">
         <v>505</v>
       </c>
@@ -5677,7 +5732,7 @@
       <c r="H21" s="5"/>
       <c r="I21" s="5"/>
     </row>
-    <row r="22" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A22" s="5" t="s">
         <v>507</v>
       </c>
@@ -5702,7 +5757,7 @@
       <c r="H22" s="5"/>
       <c r="I22" s="5"/>
     </row>
-    <row r="23" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A23" s="5" t="s">
         <v>509</v>
       </c>
@@ -5727,7 +5782,7 @@
       <c r="H23" s="5"/>
       <c r="I23" s="5"/>
     </row>
-    <row r="24" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A24" s="5" t="s">
         <v>510</v>
       </c>
@@ -5752,7 +5807,7 @@
       <c r="H24" s="5"/>
       <c r="I24" s="5"/>
     </row>
-    <row r="25" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A25" s="5" t="s">
         <v>515</v>
       </c>
@@ -5777,7 +5832,7 @@
       <c r="H25" s="5"/>
       <c r="I25" s="5"/>
     </row>
-    <row r="26" spans="1:9" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A26" s="5" t="s">
         <v>519</v>
       </c>
@@ -5802,7 +5857,7 @@
       <c r="H26" s="5"/>
       <c r="I26" s="5"/>
     </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A27" s="5" t="s">
         <v>524</v>
       </c>
@@ -5827,7 +5882,7 @@
       <c r="H27" s="5"/>
       <c r="I27" s="5"/>
     </row>
-    <row r="28" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A28" s="5" t="s">
         <v>529</v>
       </c>
@@ -5852,7 +5907,7 @@
       <c r="H28" s="5"/>
       <c r="I28" s="5"/>
     </row>
-    <row r="29" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A29" s="5" t="s">
         <v>533</v>
       </c>
@@ -5877,7 +5932,7 @@
       <c r="H29" s="5"/>
       <c r="I29" s="5"/>
     </row>
-    <row r="30" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A30" s="5" t="s">
         <v>538</v>
       </c>
@@ -5902,7 +5957,7 @@
       <c r="H30" s="5"/>
       <c r="I30" s="5"/>
     </row>
-    <row r="31" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A31" s="5" t="s">
         <v>543</v>
       </c>
@@ -5927,7 +5982,7 @@
       <c r="H31" s="5"/>
       <c r="I31" s="5"/>
     </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A32" s="5" t="s">
         <v>546</v>
       </c>
@@ -5952,7 +6007,7 @@
       <c r="H32" s="5"/>
       <c r="I32" s="5"/>
     </row>
-    <row r="33" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A33" s="5" t="s">
         <v>550</v>
       </c>
@@ -5977,7 +6032,7 @@
       <c r="H33" s="5"/>
       <c r="I33" s="5"/>
     </row>
-    <row r="34" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A34" s="5" t="s">
         <v>555</v>
       </c>
@@ -6002,7 +6057,7 @@
       <c r="H34" s="5"/>
       <c r="I34" s="5"/>
     </row>
-    <row r="35" spans="1:9" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A35" s="5" t="s">
         <v>560</v>
       </c>
@@ -6027,7 +6082,7 @@
       <c r="H35" s="5"/>
       <c r="I35" s="5"/>
     </row>
-    <row r="36" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A36" s="5" t="s">
         <v>564</v>
       </c>
@@ -6060,24 +6115,24 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A67CEC3C-A5E2-4A58-98AE-A36DD7E149E3}">
   <dimension ref="A1:I26"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="14.6640625" customWidth="1"/>
-    <col min="2" max="2" width="26.6640625" customWidth="1"/>
-    <col min="3" max="3" width="30.6640625" customWidth="1"/>
-    <col min="4" max="4" width="32.6640625" customWidth="1"/>
-    <col min="5" max="6" width="42.6640625" customWidth="1"/>
-    <col min="7" max="7" width="10.6640625" customWidth="1"/>
-    <col min="8" max="8" width="12.6640625" customWidth="1"/>
-    <col min="9" max="9" width="30.6640625" customWidth="1"/>
+    <col min="1" max="1" width="14.7109375" customWidth="1"/>
+    <col min="2" max="2" width="26.7109375" customWidth="1"/>
+    <col min="3" max="3" width="30.7109375" customWidth="1"/>
+    <col min="4" max="4" width="32.7109375" customWidth="1"/>
+    <col min="5" max="6" width="42.7109375" customWidth="1"/>
+    <col min="7" max="7" width="10.7109375" customWidth="1"/>
+    <col min="8" max="8" width="12.7109375" customWidth="1"/>
+    <col min="9" max="9" width="30.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="18" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:9" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>569</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
@@ -6085,7 +6140,7 @@
         <v>570</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>3</v>
       </c>
@@ -6093,7 +6148,7 @@
         <v>571</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>5</v>
       </c>
@@ -6101,7 +6156,7 @@
         <v>46248</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>6</v>
       </c>
@@ -6109,7 +6164,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
         <v>7</v>
       </c>
@@ -6138,7 +6193,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="8" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A8" s="5" t="s">
         <v>572</v>
       </c>
@@ -6163,7 +6218,7 @@
       <c r="H8" s="5"/>
       <c r="I8" s="5"/>
     </row>
-    <row r="9" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A9" s="5" t="s">
         <v>576</v>
       </c>
@@ -6188,7 +6243,7 @@
       <c r="H9" s="5"/>
       <c r="I9" s="5"/>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A10" s="5" t="s">
         <v>581</v>
       </c>
@@ -6213,7 +6268,7 @@
       <c r="H10" s="5"/>
       <c r="I10" s="5"/>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" s="5" t="s">
         <v>585</v>
       </c>
@@ -6238,7 +6293,7 @@
       <c r="H11" s="5"/>
       <c r="I11" s="5"/>
     </row>
-    <row r="12" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A12" s="5" t="s">
         <v>590</v>
       </c>
@@ -6263,7 +6318,7 @@
       <c r="H12" s="5"/>
       <c r="I12" s="5"/>
     </row>
-    <row r="13" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A13" s="5" t="s">
         <v>595</v>
       </c>
@@ -6288,7 +6343,7 @@
       <c r="H13" s="5"/>
       <c r="I13" s="5"/>
     </row>
-    <row r="14" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A14" s="5" t="s">
         <v>600</v>
       </c>
@@ -6313,7 +6368,7 @@
       <c r="H14" s="5"/>
       <c r="I14" s="5"/>
     </row>
-    <row r="15" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A15" s="5" t="s">
         <v>603</v>
       </c>
@@ -6338,7 +6393,7 @@
       <c r="H15" s="5"/>
       <c r="I15" s="5"/>
     </row>
-    <row r="16" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A16" s="5" t="s">
         <v>608</v>
       </c>
@@ -6363,7 +6418,7 @@
       <c r="H16" s="5"/>
       <c r="I16" s="5"/>
     </row>
-    <row r="17" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A17" s="5" t="s">
         <v>612</v>
       </c>
@@ -6388,7 +6443,7 @@
       <c r="H17" s="5"/>
       <c r="I17" s="5"/>
     </row>
-    <row r="18" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A18" s="5" t="s">
         <v>617</v>
       </c>
@@ -6413,7 +6468,7 @@
       <c r="H18" s="5"/>
       <c r="I18" s="5"/>
     </row>
-    <row r="19" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A19" s="5" t="s">
         <v>621</v>
       </c>
@@ -6438,7 +6493,7 @@
       <c r="H19" s="5"/>
       <c r="I19" s="5"/>
     </row>
-    <row r="20" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A20" s="5" t="s">
         <v>626</v>
       </c>
@@ -6463,7 +6518,7 @@
       <c r="H20" s="5"/>
       <c r="I20" s="5"/>
     </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A21" s="5" t="s">
         <v>631</v>
       </c>
@@ -6488,7 +6543,7 @@
       <c r="H21" s="5"/>
       <c r="I21" s="5"/>
     </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A22" s="5" t="s">
         <v>636</v>
       </c>
@@ -6513,7 +6568,7 @@
       <c r="H22" s="5"/>
       <c r="I22" s="5"/>
     </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A23" s="5" t="s">
         <v>641</v>
       </c>
@@ -6538,7 +6593,7 @@
       <c r="H23" s="5"/>
       <c r="I23" s="5"/>
     </row>
-    <row r="24" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A24" s="5" t="s">
         <v>643</v>
       </c>
@@ -6563,7 +6618,7 @@
       <c r="H24" s="5"/>
       <c r="I24" s="5"/>
     </row>
-    <row r="25" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A25" s="5" t="s">
         <v>648</v>
       </c>
@@ -6588,7 +6643,7 @@
       <c r="H25" s="5"/>
       <c r="I25" s="5"/>
     </row>
-    <row r="26" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A26" s="5" t="s">
         <v>652</v>
       </c>

</xml_diff>